<commit_message>
Update schedule and styling: add Wagar 107 topics, modify exam labels, and enhance table row styling for clarity
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF3F376-C720-5B48-BDA1-513AE3CE21FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5B3045-20FC-124A-859F-6343B901B603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>Review</t>
   </si>
@@ -118,24 +118,12 @@
     <t>Presentation/discussion</t>
   </si>
   <si>
-    <t>Midterm 1</t>
-  </si>
-  <si>
-    <t>Karush Kuhn Tucker and corner solutions</t>
-  </si>
-  <si>
-    <t>Midterm 2</t>
-  </si>
-  <si>
     <t>Risk, uncertainty, and scenario analysis in static models</t>
   </si>
   <si>
     <t>Infinite-horizon Bellman equation and value function iteration</t>
   </si>
   <si>
-    <t>Final</t>
-  </si>
-  <si>
     <t>Stewart &amp; Greenhalgh (1977)</t>
   </si>
   <si>
@@ -178,10 +166,25 @@
     <t>Discrete time finite horizon: formulation</t>
   </si>
   <si>
-    <t>Discrete time finite horizon: solution concepts</t>
-  </si>
-  <si>
     <t>Schlachtberger et al (2017)</t>
+  </si>
+  <si>
+    <t>Wagar 107: Review</t>
+  </si>
+  <si>
+    <t>Wagar 107: Karush Kuhn Tucker and corner solutions</t>
+  </si>
+  <si>
+    <t>Wagar 107: Discrete time finite horizon: solution concepts</t>
+  </si>
+  <si>
+    <t>Exam 1</t>
+  </si>
+  <si>
+    <t>Exam 2</t>
+  </si>
+  <si>
+    <t>Final Exam</t>
   </si>
 </sst>
 </file>
@@ -622,7 +625,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -638,7 +641,7 @@
         <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E3" s="3"/>
     </row>
@@ -652,7 +655,7 @@
         <v>46266</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -670,7 +673,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" x14ac:dyDescent="0.15">
@@ -683,10 +686,10 @@
         <v>46273</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E6" s="3"/>
     </row>
@@ -700,10 +703,10 @@
         <v>46275</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -731,10 +734,10 @@
         <v>46282</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E9" s="3"/>
     </row>
@@ -761,7 +764,7 @@
         <v>46288</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="3"/>
@@ -776,7 +779,7 @@
         <v>46289</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="13" x14ac:dyDescent="0.15">
@@ -789,7 +792,7 @@
         <v>46294</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D13" s="3"/>
     </row>
@@ -803,10 +806,10 @@
         <v>46296</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E14" s="8"/>
     </row>
@@ -833,7 +836,7 @@
         <v>46302</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="3"/>
@@ -848,7 +851,7 @@
         <v>46303</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E17" s="7"/>
     </row>
@@ -876,7 +879,7 @@
         <v>46310</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E19" s="3"/>
     </row>
@@ -917,7 +920,7 @@
         <v>46322</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="E22" s="3"/>
     </row>
@@ -931,7 +934,7 @@
         <v>46324</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="7"/>
@@ -946,7 +949,7 @@
         <v>46329</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="7"/>
@@ -959,7 +962,7 @@
         <v>46330</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="7"/>
@@ -974,7 +977,7 @@
         <v>46331</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D26" s="3"/>
     </row>
@@ -1001,7 +1004,7 @@
         <v>46338</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D28" s="3"/>
     </row>
@@ -1028,7 +1031,7 @@
         <v>46344</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="7"/>
@@ -1043,7 +1046,7 @@
         <v>46345</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>

</xml_diff>

<commit_message>
update schedule with HH paper
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -857,6 +857,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="7"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Helfand &amp; House (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="18" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A18" s="2">

</xml_diff>

<commit_message>
update ando material and schedule
</commit_message>
<xml_diff>
--- a/syllabus/AREC 615 Class Schedule.xlsx
+++ b/syllabus/AREC 615 Class Schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/judebayham/Documents/git_projects/arec-615/syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC3795DB-8C72-D24A-9076-C95C3BA28FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E021677-385C-7B41-889C-3316FB385F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,6 +54,7 @@
     <definedName name="solver_ver" localSheetId="0" hidden="1">2</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -74,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="40">
   <si>
     <t>Review</t>
   </si>
@@ -188,6 +189,12 @@
   </si>
   <si>
     <t>Kaiser and Messer Chapter 8</t>
+  </si>
+  <si>
+    <t>Ando &amp; Mallory (2012)</t>
+  </si>
+  <si>
+    <t>No class</t>
   </si>
 </sst>
 </file>
@@ -857,11 +864,6 @@
         <v>23</v>
       </c>
       <c r="E17" s="7"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Helfand &amp; House (1995)</t>
-        </is>
-      </c>
     </row>
     <row r="18" spans="1:5" ht="13" x14ac:dyDescent="0.15">
       <c r="A18" s="2">
@@ -889,10 +891,8 @@
       <c r="C19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Ando &amp; Mallory (2012)</t>
-        </is>
+      <c r="D19" t="s">
+        <v>38</v>
       </c>
       <c r="E19" s="3"/>
     </row>
@@ -906,7 +906,7 @@
         <v>46315</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="D20" s="3"/>
     </row>

</xml_diff>